<commit_message>
Atualiza SWOT: preço, experiência, investimento em outras regiões e região pouco movimentada
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-matriz-swot.xlsx
+++ b/01-matriz-swot.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Atendimento familiar dos anfitriões, elogiado pelo nome</t>
+          <t>Experiência para o consumidor: atendimento familiar, café da manhã regional, rede e jardim com orquídeas</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -507,7 +507,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Café da manhã regional, com adaptação sem glúten e sem lactose</t>
+          <t>Preço: custo de viagem e de hospedagem menor que o da região</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -524,7 +524,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Jardim com orquídeas e aves, rede em cada quarto, piscina e área social</t>
+          <t>Piscina e área social para petiscos e churrasco</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -588,7 +588,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Mudança política: a gestão atual tornou gratuita de novo a entrada da cachoeira (17/03/2025), com acesso melhorado</t>
+          <t>Mudança política: a gestão atual tornou gratuita de novo a entrada da cachoeira (17/03/2025)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Buenos Aires (Guarapari), com investimento pesado</t>
+          <t>Investimento massivo em outras regiões turísticas, como Buenos Aires (Guarapari)</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Turismo de montanha capixaba em crescimento</t>
+          <t>Pousadas de montanha em alta agora, com o turismo capixaba em crescimento</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Custo de viagem em Matilde menor que o da região</t>
+          <t>Região ainda pouco movimentada: sem congestionamento, ideal para quem busca sossego</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">

</xml_diff>